<commit_message>
Correct nine points in Finding and Removing Duplicates
The gender column has eight spellings, not six, and the solutions' country column eight, not seven. The fuzzy-match answer quotes the printed scores of 1.00 and 0.47. record_id is copied onto every duplicate, so it identifies a contact as email does, and the page, Codebook and Notes now say so. pd.to_datetime needs format="mixed" for mixed formats, or pandas reads every value in the first one's format. drop_duplicates with no subset keeps identical copies, so the advice about completeness now applies to a key. Levenshtein counts substitutions, standardizing case and punctuation catches the quiz's Acme pair, and duplicates across a split are a common cause of production failure, not the single most common.
</commit_message>
<xml_diff>
--- a/data/finding-and-removing-duplicates-and-inconsistencies--duplicate_contacts.xlsx
+++ b/data/finding-and-removing-duplicates-and-inconsistencies--duplicate_contacts.xlsx
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Row identifier (NOT unique per person)</t>
+          <t>Contact identifier, copied onto every duplicate row of that contact</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5781,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>record_id is just a row id, it is NOT a per-person key, do not dedupe on it.</t>
+          <t>record_id is copied onto each duplicate, so here it identifies a contact as well as email does. Many real systems give every row its own id, which is why a business key such as email is the safer choice.</t>
         </is>
       </c>
     </row>

</xml_diff>